<commit_message>
fix: correct country, continent, and state/province fields in VM0044 schema
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

Signed-off-by: Daniel Swid <daniel.swid@hashgraph.com>
</commit_message>
<xml_diff>
--- a/Methodology Library/Verra/Verified Carbon Standard (VCS)/VM0044 v2/VM0044 Schema.xlsx
+++ b/Methodology Library/Verra/Verified Carbon Standard (VCS)/VM0044 v2/VM0044 Schema.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10726"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CC19F7-CF7F-9B41-909E-B60638A5FBAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3879296A-61DE-FD4F-93E6-A544D959DBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-3480" yWindow="-28200" windowWidth="41060" windowHeight="28200" activeTab="3" xr2:uid="{B7272DD0-C00E-2B49-881A-D449616BA167}"/>
     <workbookView xWindow="22120" yWindow="-28200" windowWidth="25600" windowHeight="28200" activeTab="6" xr2:uid="{4ED42108-A172-AF46-A4EE-5B283497DA30}"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16968" uniqueCount="2124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16968" uniqueCount="2128">
   <si>
     <t>Project Proponent Account Registration</t>
   </si>
@@ -6732,6 +6732,18 @@
   </si>
   <si>
     <t>3 Application of Methodology</t>
+  </si>
+  <si>
+    <t>State/Province</t>
+  </si>
+  <si>
+    <t>US-CA</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>US</t>
   </si>
 </sst>
 </file>
@@ -12198,23 +12210,23 @@
         <v>21</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>2023</v>
-      </c>
-      <c r="C77" s="33" t="s">
-        <v>2023</v>
+        <v>198</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>2</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E77" s="12" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F77" s="4"/>
       <c r="G77" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>19</v>
+        <v>2126</v>
       </c>
       <c r="I77" s="4" t="s">
         <v>2</v>
@@ -12223,7 +12235,7 @@
         <v>2</v>
       </c>
       <c r="L77" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
     </row>
     <row r="78" spans="1:12" ht="16" outlineLevel="3" collapsed="1" x14ac:dyDescent="0.2">
@@ -12231,23 +12243,23 @@
         <v>21</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C78" s="4" t="s">
-        <v>2</v>
+        <v>2023</v>
+      </c>
+      <c r="C78" s="33" t="s">
+        <v>200</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E78" s="12" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F78" s="4"/>
       <c r="G78" s="4" t="s">
         <v>15</v>
       </c>
       <c r="H78" s="4" t="s">
-        <v>19</v>
+        <v>2127</v>
       </c>
       <c r="I78" s="4" t="s">
         <v>2</v>
@@ -12256,7 +12268,7 @@
         <v>2</v>
       </c>
       <c r="L78" s="4" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="79" spans="1:12" ht="16" outlineLevel="3" collapsed="1" x14ac:dyDescent="0.2">
@@ -12264,10 +12276,10 @@
         <v>21</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>16</v>
+        <v>2124</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>2</v>
+        <v>197</v>
       </c>
       <c r="D79" s="4" t="s">
         <v>203</v>
@@ -12280,7 +12292,7 @@
         <v>15</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>19</v>
+        <v>2125</v>
       </c>
       <c r="I79" s="4" t="s">
         <v>2</v>

</xml_diff>